<commit_message>
chore: pipeline update 2026-04-16 19:27
Refresh multi-sport pipeline outputs, graded report artifacts, and ticket evaluation JSON after the latest data run so published snapshots match current processing results.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ui_runner/graded_slate/2026-04-02/graded_soccer_2026-04-02.xlsx
+++ b/ui_runner/graded_slate/2026-04-02/graded_soccer_2026-04-02.xlsx
@@ -2560,7 +2560,7 @@
         <v>3.5</v>
       </c>
       <c r="G38">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H38" t="s">
         <v>273</v>
@@ -2572,7 +2572,7 @@
         <v>278</v>
       </c>
       <c r="K38">
-        <v>-2.5</v>
+        <v>-3.5</v>
       </c>
       <c r="L38">
         <v>66</v>
@@ -2832,13 +2832,10 @@
         <v>274</v>
       </c>
       <c r="J45" t="s">
-        <v>278</v>
-      </c>
-      <c r="K45">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L45">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="N45" t="s">
         <v>281</v>
@@ -4081,13 +4078,10 @@
         <v>274</v>
       </c>
       <c r="J80" t="s">
-        <v>278</v>
-      </c>
-      <c r="K80">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L80">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="N80" t="s">
         <v>281</v>
@@ -5458,13 +5452,10 @@
         <v>274</v>
       </c>
       <c r="J119" t="s">
-        <v>278</v>
-      </c>
-      <c r="K119">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L119">
-        <v>35.1</v>
+        <v>0</v>
       </c>
       <c r="N119" t="s">
         <v>281</v>
@@ -6135,13 +6126,10 @@
         <v>275</v>
       </c>
       <c r="J138" t="s">
-        <v>278</v>
-      </c>
-      <c r="K138">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L138">
-        <v>31.4925</v>
+        <v>0</v>
       </c>
       <c r="N138" t="s">
         <v>281</v>
@@ -6176,13 +6164,10 @@
         <v>275</v>
       </c>
       <c r="J139" t="s">
-        <v>278</v>
-      </c>
-      <c r="K139">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L139">
-        <v>31.4925</v>
+        <v>0</v>
       </c>
       <c r="N139" t="s">
         <v>281</v>
@@ -6217,13 +6202,10 @@
         <v>275</v>
       </c>
       <c r="J140" t="s">
-        <v>278</v>
-      </c>
-      <c r="K140">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L140">
-        <v>42.075</v>
+        <v>0</v>
       </c>
       <c r="N140" t="s">
         <v>281</v>
@@ -6334,13 +6316,10 @@
         <v>275</v>
       </c>
       <c r="J143" t="s">
-        <v>278</v>
-      </c>
-      <c r="K143">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L143">
-        <v>35.95500000000001</v>
+        <v>0</v>
       </c>
       <c r="N143" t="s">
         <v>281</v>
@@ -6941,13 +6920,10 @@
         <v>275</v>
       </c>
       <c r="J160" t="s">
-        <v>278</v>
-      </c>
-      <c r="K160">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L160">
-        <v>31.4925</v>
+        <v>0</v>
       </c>
       <c r="N160" t="s">
         <v>281</v>
@@ -7204,13 +7180,10 @@
         <v>276</v>
       </c>
       <c r="J167" t="s">
-        <v>278</v>
-      </c>
-      <c r="K167">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L167">
-        <v>36.575</v>
+        <v>0</v>
       </c>
       <c r="N167" t="s">
         <v>281</v>
@@ -7461,13 +7434,10 @@
         <v>276</v>
       </c>
       <c r="J174" t="s">
-        <v>278</v>
-      </c>
-      <c r="K174">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L174">
-        <v>25.935</v>
+        <v>0</v>
       </c>
       <c r="N174" t="s">
         <v>281</v>
@@ -7572,13 +7542,10 @@
         <v>276</v>
       </c>
       <c r="J177" t="s">
-        <v>278</v>
-      </c>
-      <c r="K177">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L177">
-        <v>25.935</v>
+        <v>0</v>
       </c>
       <c r="N177" t="s">
         <v>281</v>
@@ -8628,13 +8595,10 @@
         <v>276</v>
       </c>
       <c r="J207" t="s">
-        <v>278</v>
-      </c>
-      <c r="K207">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L207">
-        <v>24.57</v>
+        <v>0</v>
       </c>
       <c r="N207" t="s">
         <v>281</v>
@@ -9148,13 +9112,10 @@
         <v>277</v>
       </c>
       <c r="J221" t="s">
-        <v>278</v>
-      </c>
-      <c r="K221">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L221">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N221" t="s">
         <v>281</v>
@@ -9405,13 +9366,10 @@
         <v>277</v>
       </c>
       <c r="J228" t="s">
-        <v>278</v>
-      </c>
-      <c r="K228">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L228">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N228" t="s">
         <v>281</v>
@@ -9551,13 +9509,10 @@
         <v>277</v>
       </c>
       <c r="J232" t="s">
-        <v>278</v>
-      </c>
-      <c r="K232">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L232">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N232" t="s">
         <v>281</v>
@@ -10432,13 +10387,10 @@
         <v>277</v>
       </c>
       <c r="J257" t="s">
-        <v>278</v>
-      </c>
-      <c r="K257">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L257">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N257" t="s">
         <v>281</v>
@@ -10473,13 +10425,10 @@
         <v>277</v>
       </c>
       <c r="J258" t="s">
-        <v>278</v>
-      </c>
-      <c r="K258">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L258">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N258" t="s">
         <v>281</v>
@@ -10549,13 +10498,10 @@
         <v>277</v>
       </c>
       <c r="J260" t="s">
-        <v>278</v>
-      </c>
-      <c r="K260">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L260">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N260" t="s">
         <v>281</v>
@@ -10631,13 +10577,10 @@
         <v>277</v>
       </c>
       <c r="J262" t="s">
-        <v>278</v>
-      </c>
-      <c r="K262">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L262">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N262" t="s">
         <v>281</v>
@@ -10672,13 +10615,10 @@
         <v>277</v>
       </c>
       <c r="J263" t="s">
-        <v>278</v>
-      </c>
-      <c r="K263">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L263">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N263" t="s">
         <v>281</v>
@@ -10713,13 +10653,10 @@
         <v>277</v>
       </c>
       <c r="J264" t="s">
-        <v>278</v>
-      </c>
-      <c r="K264">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L264">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N264" t="s">
         <v>281</v>
@@ -10830,13 +10767,10 @@
         <v>277</v>
       </c>
       <c r="J267" t="s">
-        <v>278</v>
-      </c>
-      <c r="K267">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L267">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N267" t="s">
         <v>281</v>
@@ -10871,13 +10805,10 @@
         <v>277</v>
       </c>
       <c r="J268" t="s">
-        <v>278</v>
-      </c>
-      <c r="K268">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L268">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N268" t="s">
         <v>281</v>
@@ -11023,13 +10954,10 @@
         <v>277</v>
       </c>
       <c r="J272" t="s">
-        <v>278</v>
-      </c>
-      <c r="K272">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L272">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N272" t="s">
         <v>281</v>
@@ -11064,13 +10992,10 @@
         <v>277</v>
       </c>
       <c r="J273" t="s">
-        <v>278</v>
-      </c>
-      <c r="K273">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L273">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N273" t="s">
         <v>281</v>
@@ -11140,13 +11065,10 @@
         <v>277</v>
       </c>
       <c r="J275" t="s">
-        <v>278</v>
-      </c>
-      <c r="K275">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L275">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N275" t="s">
         <v>281</v>
@@ -11181,13 +11103,10 @@
         <v>277</v>
       </c>
       <c r="J276" t="s">
-        <v>278</v>
-      </c>
-      <c r="K276">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L276">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N276" t="s">
         <v>281</v>
@@ -11537,13 +11456,10 @@
         <v>277</v>
       </c>
       <c r="J286" t="s">
-        <v>278</v>
-      </c>
-      <c r="K286">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L286">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N286" t="s">
         <v>281</v>
@@ -11613,13 +11529,10 @@
         <v>277</v>
       </c>
       <c r="J288" t="s">
-        <v>278</v>
-      </c>
-      <c r="K288">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L288">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N288" t="s">
         <v>281</v>
@@ -11835,13 +11748,10 @@
         <v>277</v>
       </c>
       <c r="J294" t="s">
-        <v>278</v>
-      </c>
-      <c r="K294">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L294">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N294" t="s">
         <v>281</v>
@@ -11987,13 +11897,10 @@
         <v>277</v>
       </c>
       <c r="J298" t="s">
-        <v>278</v>
-      </c>
-      <c r="K298">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L298">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N298" t="s">
         <v>281</v>
@@ -12028,13 +11935,10 @@
         <v>277</v>
       </c>
       <c r="J299" t="s">
-        <v>278</v>
-      </c>
-      <c r="K299">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L299">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N299" t="s">
         <v>281</v>
@@ -12069,13 +11973,10 @@
         <v>277</v>
       </c>
       <c r="J300" t="s">
-        <v>278</v>
-      </c>
-      <c r="K300">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L300">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N300" t="s">
         <v>281</v>
@@ -12110,13 +12011,10 @@
         <v>277</v>
       </c>
       <c r="J301" t="s">
-        <v>278</v>
-      </c>
-      <c r="K301">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L301">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N301" t="s">
         <v>281</v>
@@ -12186,13 +12084,10 @@
         <v>277</v>
       </c>
       <c r="J303" t="s">
-        <v>278</v>
-      </c>
-      <c r="K303">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L303">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N303" t="s">
         <v>281</v>
@@ -12227,13 +12122,10 @@
         <v>277</v>
       </c>
       <c r="J304" t="s">
-        <v>278</v>
-      </c>
-      <c r="K304">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L304">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N304" t="s">
         <v>281</v>
@@ -12268,13 +12160,10 @@
         <v>277</v>
       </c>
       <c r="J305" t="s">
-        <v>278</v>
-      </c>
-      <c r="K305">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L305">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N305" t="s">
         <v>281</v>
@@ -12916,13 +12805,10 @@
         <v>277</v>
       </c>
       <c r="J323" t="s">
-        <v>278</v>
-      </c>
-      <c r="K323">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L323">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N323" t="s">
         <v>281</v>
@@ -12992,13 +12878,10 @@
         <v>277</v>
       </c>
       <c r="J325" t="s">
-        <v>278</v>
-      </c>
-      <c r="K325">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L325">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N325" t="s">
         <v>281</v>
@@ -13138,13 +13021,10 @@
         <v>277</v>
       </c>
       <c r="J329" t="s">
-        <v>278</v>
-      </c>
-      <c r="K329">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L329">
-        <v>26.125</v>
+        <v>0</v>
       </c>
       <c r="N329" t="s">
         <v>281</v>
@@ -13284,13 +13164,10 @@
         <v>277</v>
       </c>
       <c r="J333" t="s">
-        <v>279</v>
-      </c>
-      <c r="K333">
-        <v>2</v>
+        <v>280</v>
       </c>
       <c r="L333">
-        <v>31.95</v>
+        <v>0</v>
       </c>
       <c r="N333" t="s">
         <v>281</v>
@@ -13862,13 +13739,10 @@
         <v>277</v>
       </c>
       <c r="J349" t="s">
-        <v>278</v>
-      </c>
-      <c r="K349">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L349">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N349" t="s">
         <v>281</v>
@@ -13944,13 +13818,10 @@
         <v>277</v>
       </c>
       <c r="J351" t="s">
-        <v>278</v>
-      </c>
-      <c r="K351">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L351">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N351" t="s">
         <v>281</v>
@@ -13985,13 +13856,10 @@
         <v>277</v>
       </c>
       <c r="J352" t="s">
-        <v>278</v>
-      </c>
-      <c r="K352">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L352">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="N352" t="s">
         <v>281</v>
@@ -16377,13 +16245,10 @@
         <v>277</v>
       </c>
       <c r="J420" t="s">
-        <v>278</v>
-      </c>
-      <c r="K420">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L420">
-        <v>26.125</v>
+        <v>0</v>
       </c>
       <c r="N420" t="s">
         <v>281</v>
@@ -16418,13 +16283,10 @@
         <v>277</v>
       </c>
       <c r="J421" t="s">
-        <v>279</v>
-      </c>
-      <c r="K421">
-        <v>1.5</v>
+        <v>280</v>
       </c>
       <c r="L421">
-        <v>31.825</v>
+        <v>0</v>
       </c>
       <c r="N421" t="s">
         <v>281</v>
@@ -17253,13 +17115,10 @@
         <v>277</v>
       </c>
       <c r="J444" t="s">
-        <v>278</v>
-      </c>
-      <c r="K444">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L444">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N444" t="s">
         <v>281</v>
@@ -17504,13 +17363,10 @@
         <v>277</v>
       </c>
       <c r="J451" t="s">
-        <v>278</v>
-      </c>
-      <c r="K451">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L451">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N451" t="s">
         <v>281</v>
@@ -17545,13 +17401,10 @@
         <v>277</v>
       </c>
       <c r="J452" t="s">
-        <v>278</v>
-      </c>
-      <c r="K452">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L452">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N452" t="s">
         <v>281</v>
@@ -17586,13 +17439,10 @@
         <v>277</v>
       </c>
       <c r="J453" t="s">
-        <v>278</v>
-      </c>
-      <c r="K453">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L453">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N453" t="s">
         <v>281</v>
@@ -17662,13 +17512,10 @@
         <v>277</v>
       </c>
       <c r="J455" t="s">
-        <v>278</v>
-      </c>
-      <c r="K455">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L455">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N455" t="s">
         <v>281</v>
@@ -17703,13 +17550,10 @@
         <v>277</v>
       </c>
       <c r="J456" t="s">
-        <v>278</v>
-      </c>
-      <c r="K456">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L456">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N456" t="s">
         <v>281</v>
@@ -17814,13 +17658,10 @@
         <v>277</v>
       </c>
       <c r="J459" t="s">
-        <v>278</v>
-      </c>
-      <c r="K459">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L459">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N459" t="s">
         <v>281</v>
@@ -17890,13 +17731,10 @@
         <v>277</v>
       </c>
       <c r="J461" t="s">
-        <v>278</v>
-      </c>
-      <c r="K461">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L461">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N461" t="s">
         <v>281</v>
@@ -17931,13 +17769,10 @@
         <v>277</v>
       </c>
       <c r="J462" t="s">
-        <v>278</v>
-      </c>
-      <c r="K462">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L462">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N462" t="s">
         <v>281</v>
@@ -17972,13 +17807,10 @@
         <v>277</v>
       </c>
       <c r="J463" t="s">
-        <v>278</v>
-      </c>
-      <c r="K463">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L463">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N463" t="s">
         <v>281</v>
@@ -18083,13 +17915,10 @@
         <v>277</v>
       </c>
       <c r="J466" t="s">
-        <v>278</v>
-      </c>
-      <c r="K466">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L466">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N466" t="s">
         <v>281</v>
@@ -18124,13 +17953,10 @@
         <v>277</v>
       </c>
       <c r="J467" t="s">
-        <v>278</v>
-      </c>
-      <c r="K467">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L467">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N467" t="s">
         <v>281</v>
@@ -18165,13 +17991,10 @@
         <v>277</v>
       </c>
       <c r="J468" t="s">
-        <v>278</v>
-      </c>
-      <c r="K468">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L468">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N468" t="s">
         <v>281</v>
@@ -18206,13 +18029,10 @@
         <v>277</v>
       </c>
       <c r="J469" t="s">
-        <v>278</v>
-      </c>
-      <c r="K469">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L469">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N469" t="s">
         <v>281</v>
@@ -18247,13 +18067,10 @@
         <v>277</v>
       </c>
       <c r="J470" t="s">
-        <v>278</v>
-      </c>
-      <c r="K470">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L470">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N470" t="s">
         <v>281</v>
@@ -18288,13 +18105,10 @@
         <v>277</v>
       </c>
       <c r="J471" t="s">
-        <v>278</v>
-      </c>
-      <c r="K471">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L471">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N471" t="s">
         <v>281</v>
@@ -18405,13 +18219,10 @@
         <v>277</v>
       </c>
       <c r="J474" t="s">
-        <v>278</v>
-      </c>
-      <c r="K474">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L474">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N474" t="s">
         <v>281</v>
@@ -18481,13 +18292,10 @@
         <v>277</v>
       </c>
       <c r="J476" t="s">
-        <v>278</v>
-      </c>
-      <c r="K476">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L476">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N476" t="s">
         <v>281</v>
@@ -18522,13 +18330,10 @@
         <v>277</v>
       </c>
       <c r="J477" t="s">
-        <v>278</v>
-      </c>
-      <c r="K477">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L477">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N477" t="s">
         <v>281</v>
@@ -18563,13 +18368,10 @@
         <v>277</v>
       </c>
       <c r="J478" t="s">
-        <v>278</v>
-      </c>
-      <c r="K478">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L478">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N478" t="s">
         <v>281</v>
@@ -19409,13 +19211,10 @@
         <v>277</v>
       </c>
       <c r="J502" t="s">
-        <v>278</v>
-      </c>
-      <c r="K502">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L502">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N502" t="s">
         <v>281</v>
@@ -20092,13 +19891,10 @@
         <v>277</v>
       </c>
       <c r="J521" t="s">
-        <v>278</v>
-      </c>
-      <c r="K521">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L521">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N521" t="s">
         <v>281</v>
@@ -20343,13 +20139,10 @@
         <v>277</v>
       </c>
       <c r="J528" t="s">
-        <v>278</v>
-      </c>
-      <c r="K528">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L528">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N528" t="s">
         <v>281</v>
@@ -20384,13 +20177,10 @@
         <v>277</v>
       </c>
       <c r="J529" t="s">
-        <v>278</v>
-      </c>
-      <c r="K529">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L529">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N529" t="s">
         <v>281</v>
@@ -20425,13 +20215,10 @@
         <v>277</v>
       </c>
       <c r="J530" t="s">
-        <v>278</v>
-      </c>
-      <c r="K530">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L530">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N530" t="s">
         <v>281</v>
@@ -20501,13 +20288,10 @@
         <v>277</v>
       </c>
       <c r="J532" t="s">
-        <v>278</v>
-      </c>
-      <c r="K532">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L532">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N532" t="s">
         <v>281</v>
@@ -20542,13 +20326,10 @@
         <v>277</v>
       </c>
       <c r="J533" t="s">
-        <v>278</v>
-      </c>
-      <c r="K533">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L533">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N533" t="s">
         <v>281</v>
@@ -20583,13 +20364,10 @@
         <v>277</v>
       </c>
       <c r="J534" t="s">
-        <v>278</v>
-      </c>
-      <c r="K534">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L534">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N534" t="s">
         <v>281</v>
@@ -20624,13 +20402,10 @@
         <v>277</v>
       </c>
       <c r="J535" t="s">
-        <v>278</v>
-      </c>
-      <c r="K535">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L535">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N535" t="s">
         <v>281</v>
@@ -21266,13 +21041,10 @@
         <v>277</v>
       </c>
       <c r="J553" t="s">
-        <v>278</v>
-      </c>
-      <c r="K553">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L553">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N553" t="s">
         <v>281</v>
@@ -21377,13 +21149,10 @@
         <v>277</v>
       </c>
       <c r="J556" t="s">
-        <v>278</v>
-      </c>
-      <c r="K556">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L556">
-        <v>27.5</v>
+        <v>0</v>
       </c>
       <c r="N556" t="s">
         <v>281</v>
@@ -21838,13 +21607,10 @@
         <v>277</v>
       </c>
       <c r="J569" t="s">
-        <v>278</v>
-      </c>
-      <c r="K569">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L569">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N569" t="s">
         <v>281</v>
@@ -21914,13 +21680,10 @@
         <v>277</v>
       </c>
       <c r="J571" t="s">
-        <v>278</v>
-      </c>
-      <c r="K571">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L571">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N571" t="s">
         <v>281</v>
@@ -21955,13 +21718,10 @@
         <v>277</v>
       </c>
       <c r="J572" t="s">
-        <v>278</v>
-      </c>
-      <c r="K572">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L572">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N572" t="s">
         <v>281</v>
@@ -22031,13 +21791,10 @@
         <v>277</v>
       </c>
       <c r="J574" t="s">
-        <v>278</v>
-      </c>
-      <c r="K574">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L574">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N574" t="s">
         <v>281</v>
@@ -22072,13 +21829,10 @@
         <v>277</v>
       </c>
       <c r="J575" t="s">
-        <v>278</v>
-      </c>
-      <c r="K575">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L575">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N575" t="s">
         <v>281</v>
@@ -22113,13 +21867,10 @@
         <v>277</v>
       </c>
       <c r="J576" t="s">
-        <v>278</v>
-      </c>
-      <c r="K576">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L576">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N576" t="s">
         <v>281</v>
@@ -22154,13 +21905,10 @@
         <v>277</v>
       </c>
       <c r="J577" t="s">
-        <v>278</v>
-      </c>
-      <c r="K577">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L577">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N577" t="s">
         <v>281</v>
@@ -22195,13 +21943,10 @@
         <v>277</v>
       </c>
       <c r="J578" t="s">
-        <v>278</v>
-      </c>
-      <c r="K578">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L578">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N578" t="s">
         <v>281</v>
@@ -22236,13 +21981,10 @@
         <v>277</v>
       </c>
       <c r="J579" t="s">
-        <v>278</v>
-      </c>
-      <c r="K579">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L579">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N579" t="s">
         <v>281</v>
@@ -22312,13 +22054,10 @@
         <v>277</v>
       </c>
       <c r="J581" t="s">
-        <v>278</v>
-      </c>
-      <c r="K581">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L581">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N581" t="s">
         <v>281</v>
@@ -22353,13 +22092,10 @@
         <v>277</v>
       </c>
       <c r="J582" t="s">
-        <v>278</v>
-      </c>
-      <c r="K582">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L582">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N582" t="s">
         <v>281</v>
@@ -22394,13 +22130,10 @@
         <v>277</v>
       </c>
       <c r="J583" t="s">
-        <v>278</v>
-      </c>
-      <c r="K583">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L583">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N583" t="s">
         <v>281</v>
@@ -22435,13 +22168,10 @@
         <v>277</v>
       </c>
       <c r="J584" t="s">
-        <v>278</v>
-      </c>
-      <c r="K584">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L584">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N584" t="s">
         <v>281</v>
@@ -22476,13 +22206,10 @@
         <v>277</v>
       </c>
       <c r="J585" t="s">
-        <v>278</v>
-      </c>
-      <c r="K585">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L585">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N585" t="s">
         <v>281</v>
@@ -22517,13 +22244,10 @@
         <v>277</v>
       </c>
       <c r="J586" t="s">
-        <v>278</v>
-      </c>
-      <c r="K586">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L586">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N586" t="s">
         <v>281</v>
@@ -22558,13 +22282,10 @@
         <v>277</v>
       </c>
       <c r="J587" t="s">
-        <v>278</v>
-      </c>
-      <c r="K587">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L587">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N587" t="s">
         <v>281</v>
@@ -22634,13 +22355,10 @@
         <v>277</v>
       </c>
       <c r="J589" t="s">
-        <v>278</v>
-      </c>
-      <c r="K589">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L589">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N589" t="s">
         <v>281</v>
@@ -22675,13 +22393,10 @@
         <v>277</v>
       </c>
       <c r="J590" t="s">
-        <v>278</v>
-      </c>
-      <c r="K590">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L590">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N590" t="s">
         <v>281</v>
@@ -22716,13 +22431,10 @@
         <v>277</v>
       </c>
       <c r="J591" t="s">
-        <v>278</v>
-      </c>
-      <c r="K591">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L591">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N591" t="s">
         <v>281</v>
@@ -22757,13 +22469,10 @@
         <v>277</v>
       </c>
       <c r="J592" t="s">
-        <v>278</v>
-      </c>
-      <c r="K592">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L592">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N592" t="s">
         <v>281</v>
@@ -22798,13 +22507,10 @@
         <v>277</v>
       </c>
       <c r="J593" t="s">
-        <v>278</v>
-      </c>
-      <c r="K593">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L593">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N593" t="s">
         <v>281</v>
@@ -22839,13 +22545,10 @@
         <v>277</v>
       </c>
       <c r="J594" t="s">
-        <v>278</v>
-      </c>
-      <c r="K594">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L594">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N594" t="s">
         <v>281</v>
@@ -23930,13 +23633,10 @@
         <v>277</v>
       </c>
       <c r="J625" t="s">
-        <v>278</v>
-      </c>
-      <c r="K625">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L625">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N625" t="s">
         <v>281</v>
@@ -23971,13 +23671,10 @@
         <v>277</v>
       </c>
       <c r="J626" t="s">
-        <v>278</v>
-      </c>
-      <c r="K626">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L626">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N626" t="s">
         <v>281</v>
@@ -24047,13 +23744,10 @@
         <v>277</v>
       </c>
       <c r="J628" t="s">
-        <v>278</v>
-      </c>
-      <c r="K628">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L628">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="N628" t="s">
         <v>281</v>
@@ -24088,13 +23782,10 @@
         <v>277</v>
       </c>
       <c r="J629" t="s">
-        <v>278</v>
-      </c>
-      <c r="K629">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L629">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N629" t="s">
         <v>281</v>
@@ -24199,13 +23890,10 @@
         <v>277</v>
       </c>
       <c r="J632" t="s">
-        <v>278</v>
-      </c>
-      <c r="K632">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L632">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N632" t="s">
         <v>281</v>
@@ -24240,13 +23928,10 @@
         <v>277</v>
       </c>
       <c r="J633" t="s">
-        <v>278</v>
-      </c>
-      <c r="K633">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L633">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N633" t="s">
         <v>281</v>
@@ -24357,13 +24042,10 @@
         <v>277</v>
       </c>
       <c r="J636" t="s">
-        <v>278</v>
-      </c>
-      <c r="K636">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L636">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N636" t="s">
         <v>281</v>
@@ -24433,13 +24115,10 @@
         <v>277</v>
       </c>
       <c r="J638" t="s">
-        <v>278</v>
-      </c>
-      <c r="K638">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L638">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N638" t="s">
         <v>281</v>
@@ -24474,13 +24153,10 @@
         <v>277</v>
       </c>
       <c r="J639" t="s">
-        <v>278</v>
-      </c>
-      <c r="K639">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L639">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N639" t="s">
         <v>281</v>
@@ -24515,13 +24191,10 @@
         <v>277</v>
       </c>
       <c r="J640" t="s">
-        <v>278</v>
-      </c>
-      <c r="K640">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L640">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N640" t="s">
         <v>281</v>
@@ -24591,13 +24264,10 @@
         <v>277</v>
       </c>
       <c r="J642" t="s">
-        <v>278</v>
-      </c>
-      <c r="K642">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L642">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N642" t="s">
         <v>281</v>
@@ -24632,13 +24302,10 @@
         <v>277</v>
       </c>
       <c r="J643" t="s">
-        <v>278</v>
-      </c>
-      <c r="K643">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L643">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N643" t="s">
         <v>281</v>
@@ -24743,13 +24410,10 @@
         <v>277</v>
       </c>
       <c r="J646" t="s">
-        <v>278</v>
-      </c>
-      <c r="K646">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L646">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N646" t="s">
         <v>281</v>
@@ -24819,13 +24483,10 @@
         <v>277</v>
       </c>
       <c r="J648" t="s">
-        <v>278</v>
-      </c>
-      <c r="K648">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L648">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N648" t="s">
         <v>281</v>
@@ -24860,13 +24521,10 @@
         <v>277</v>
       </c>
       <c r="J649" t="s">
-        <v>278</v>
-      </c>
-      <c r="K649">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L649">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N649" t="s">
         <v>281</v>
@@ -24936,13 +24594,10 @@
         <v>277</v>
       </c>
       <c r="J651" t="s">
-        <v>278</v>
-      </c>
-      <c r="K651">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L651">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N651" t="s">
         <v>281</v>
@@ -24977,13 +24632,10 @@
         <v>277</v>
       </c>
       <c r="J652" t="s">
-        <v>278</v>
-      </c>
-      <c r="K652">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L652">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N652" t="s">
         <v>281</v>
@@ -25053,13 +24705,10 @@
         <v>277</v>
       </c>
       <c r="J654" t="s">
-        <v>278</v>
-      </c>
-      <c r="K654">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L654">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N654" t="s">
         <v>281</v>
@@ -25094,13 +24743,10 @@
         <v>277</v>
       </c>
       <c r="J655" t="s">
-        <v>278</v>
-      </c>
-      <c r="K655">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L655">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N655" t="s">
         <v>281</v>
@@ -25135,13 +24781,10 @@
         <v>277</v>
       </c>
       <c r="J656" t="s">
-        <v>278</v>
-      </c>
-      <c r="K656">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L656">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N656" t="s">
         <v>281</v>
@@ -25211,13 +24854,10 @@
         <v>277</v>
       </c>
       <c r="J658" t="s">
-        <v>278</v>
-      </c>
-      <c r="K658">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L658">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N658" t="s">
         <v>281</v>
@@ -25252,13 +24892,10 @@
         <v>277</v>
       </c>
       <c r="J659" t="s">
-        <v>278</v>
-      </c>
-      <c r="K659">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L659">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N659" t="s">
         <v>281</v>
@@ -25334,13 +24971,10 @@
         <v>277</v>
       </c>
       <c r="J661" t="s">
-        <v>278</v>
-      </c>
-      <c r="K661">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L661">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N661" t="s">
         <v>281</v>
@@ -25375,13 +25009,10 @@
         <v>277</v>
       </c>
       <c r="J662" t="s">
-        <v>278</v>
-      </c>
-      <c r="K662">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L662">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N662" t="s">
         <v>281</v>
@@ -26898,13 +26529,10 @@
         <v>277</v>
       </c>
       <c r="J705" t="s">
-        <v>278</v>
-      </c>
-      <c r="K705">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L705">
-        <v>24.75</v>
+        <v>0</v>
       </c>
       <c r="N705" t="s">
         <v>281</v>
@@ -27149,13 +26777,10 @@
         <v>277</v>
       </c>
       <c r="J712" t="s">
-        <v>278</v>
-      </c>
-      <c r="K712">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L712">
-        <v>22.325</v>
+        <v>0</v>
       </c>
       <c r="N712" t="s">
         <v>281</v>
@@ -27330,13 +26955,10 @@
         <v>277</v>
       </c>
       <c r="J717" t="s">
-        <v>278</v>
-      </c>
-      <c r="K717">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L717">
-        <v>27.5</v>
+        <v>0</v>
       </c>
       <c r="N717" t="s">
         <v>281</v>
@@ -27371,13 +26993,10 @@
         <v>277</v>
       </c>
       <c r="J718" t="s">
-        <v>278</v>
-      </c>
-      <c r="K718">
-        <v>-2.5</v>
+        <v>280</v>
       </c>
       <c r="L718">
-        <v>26.125</v>
+        <v>0</v>
       </c>
       <c r="N718" t="s">
         <v>281</v>
@@ -28007,13 +27626,10 @@
         <v>277</v>
       </c>
       <c r="J736" t="s">
-        <v>278</v>
-      </c>
-      <c r="K736">
-        <v>-3.5</v>
+        <v>280</v>
       </c>
       <c r="L736">
-        <v>26.125</v>
+        <v>0</v>
       </c>
       <c r="N736" t="s">
         <v>281</v>
@@ -32464,13 +32080,10 @@
         <v>277</v>
       </c>
       <c r="J863" t="s">
-        <v>278</v>
-      </c>
-      <c r="K863">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L863">
-        <v>17.55</v>
+        <v>0</v>
       </c>
       <c r="N863" t="s">
         <v>281</v>
@@ -32540,13 +32153,10 @@
         <v>277</v>
       </c>
       <c r="J865" t="s">
-        <v>278</v>
-      </c>
-      <c r="K865">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L865">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="N865" t="s">
         <v>281</v>
@@ -32762,13 +32372,10 @@
         <v>277</v>
       </c>
       <c r="J871" t="s">
-        <v>278</v>
-      </c>
-      <c r="K871">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L871">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N871" t="s">
         <v>281</v>
@@ -32978,13 +32585,10 @@
         <v>277</v>
       </c>
       <c r="J877" t="s">
-        <v>278</v>
-      </c>
-      <c r="K877">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L877">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="N877" t="s">
         <v>281</v>
@@ -33124,13 +32728,10 @@
         <v>277</v>
       </c>
       <c r="J881" t="s">
-        <v>278</v>
-      </c>
-      <c r="K881">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L881">
-        <v>18.525</v>
+        <v>0</v>
       </c>
       <c r="N881" t="s">
         <v>281</v>
@@ -33200,13 +32801,10 @@
         <v>277</v>
       </c>
       <c r="J883" t="s">
-        <v>278</v>
-      </c>
-      <c r="K883">
-        <v>-0.5</v>
+        <v>280</v>
       </c>
       <c r="L883">
-        <v>19.5</v>
+        <v>0</v>
       </c>
       <c r="N883" t="s">
         <v>281</v>
@@ -33486,13 +33084,10 @@
         <v>277</v>
       </c>
       <c r="J891" t="s">
-        <v>278</v>
-      </c>
-      <c r="K891">
-        <v>-1.5</v>
+        <v>280</v>
       </c>
       <c r="L891">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="N891" t="s">
         <v>281</v>

</xml_diff>